<commit_message>
Backend robustness improvements and formula integration
- Refactored backend logic to make the ExcelFormulaEngine more robust and consistent across input files.

- Integrated formula mappings for all technoeconomic and fuel input sheets.

- The Design Capital Structure section remains pending and will be implemented in a later update.

- Temporarily included Rwanda example input files with populated values for testing and validation purposes.
</commit_message>
<xml_diff>
--- a/backend/{templates}/fuel-financial-inputs-{template}.xlsx
+++ b/backend/{templates}/fuel-financial-inputs-{template}.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agarr\OneDrive\Escritorio\IIT\CC-WBT\backend\{templates}\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/CC-WBT/backend/{templates}/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CD95B9B-1AFB-41C2-858E-4F8E1A8D8AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Electricity" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Add new templates with updated format
- Loaded new templates with the adjusted and standardized format
</commit_message>
<xml_diff>
--- a/backend/{templates}/fuel-financial-inputs-{template}.xlsx
+++ b/backend/{templates}/fuel-financial-inputs-{template}.xlsx
@@ -1,24 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29714"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/CC-WBT/backend/{templates}/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pduen\Documents\GitHub\pre-ICCPT\CC-WBT\backend\{templates}\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{7CD95B9B-1AFB-41C2-858E-4F8E1A8D8AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3D77BA0-5D01-4B09-935B-6F2CD7D34744}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DE70EF9A-A9A2-4689-8E49-44C66F24C432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Electricity" sheetId="1" r:id="rId1"/>
     <sheet name="LPG" sheetId="2" r:id="rId2"/>
     <sheet name="Carbon Credits" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191028" iterate="1"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -83,7 +86,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -127,7 +133,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -146,8 +152,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -170,11 +182,56 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -192,7 +249,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -531,12 +597,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja1"/>
   <dimension ref="A1:AQ4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="34.81640625" customWidth="1"/>
+    <col min="1" max="1" width="34.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:43" ht="15.6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -667,138 +733,138 @@
         <v>2060</v>
       </c>
     </row>
-    <row r="2" spans="1:43" ht="16" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:43" ht="15.6">
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="6">
-        <v>0</v>
-      </c>
-      <c r="D2" s="6">
-        <v>0</v>
-      </c>
-      <c r="E2" s="6">
-        <v>0</v>
-      </c>
-      <c r="F2" s="6">
-        <v>0</v>
-      </c>
-      <c r="G2" s="6">
-        <v>0</v>
-      </c>
-      <c r="H2" s="6">
-        <v>0</v>
-      </c>
-      <c r="I2" s="6">
-        <v>0</v>
-      </c>
-      <c r="J2" s="6">
-        <v>0</v>
-      </c>
-      <c r="K2" s="6">
-        <v>0</v>
-      </c>
-      <c r="L2" s="6">
-        <v>0</v>
-      </c>
-      <c r="M2" s="6">
-        <v>0</v>
-      </c>
-      <c r="N2" s="6">
-        <v>0</v>
-      </c>
-      <c r="O2" s="6">
-        <v>0</v>
-      </c>
-      <c r="P2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="6">
-        <v>0</v>
-      </c>
-      <c r="R2" s="6">
-        <v>0</v>
-      </c>
-      <c r="S2" s="6">
-        <v>0</v>
-      </c>
-      <c r="T2" s="6">
-        <v>0</v>
-      </c>
-      <c r="U2" s="6">
-        <v>0</v>
-      </c>
-      <c r="V2" s="6">
-        <v>0</v>
-      </c>
-      <c r="W2" s="6">
-        <v>0</v>
-      </c>
-      <c r="X2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AF2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AG2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AH2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AI2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AJ2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AK2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AL2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AM2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AN2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AO2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AP2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AQ2" s="6">
+      <c r="C2" s="7">
+        <v>0</v>
+      </c>
+      <c r="D2" s="7">
+        <v>0</v>
+      </c>
+      <c r="E2" s="7">
+        <v>0</v>
+      </c>
+      <c r="F2" s="7">
+        <v>0</v>
+      </c>
+      <c r="G2" s="7">
+        <v>0</v>
+      </c>
+      <c r="H2" s="7">
+        <v>0</v>
+      </c>
+      <c r="I2" s="7">
+        <v>0</v>
+      </c>
+      <c r="J2" s="7">
+        <v>0</v>
+      </c>
+      <c r="K2" s="7">
+        <v>0</v>
+      </c>
+      <c r="L2" s="7">
+        <v>0</v>
+      </c>
+      <c r="M2" s="7">
+        <v>0</v>
+      </c>
+      <c r="N2" s="7">
+        <v>0</v>
+      </c>
+      <c r="O2" s="7">
+        <v>0</v>
+      </c>
+      <c r="P2" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="7">
+        <v>0</v>
+      </c>
+      <c r="R2" s="7">
+        <v>0</v>
+      </c>
+      <c r="S2" s="7">
+        <v>0</v>
+      </c>
+      <c r="T2" s="7">
+        <v>0</v>
+      </c>
+      <c r="U2" s="7">
+        <v>0</v>
+      </c>
+      <c r="V2" s="7">
+        <v>0</v>
+      </c>
+      <c r="W2" s="7">
+        <v>0</v>
+      </c>
+      <c r="X2" s="7">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="7">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AD2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AG2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AH2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AI2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AJ2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AK2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AL2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AM2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AN2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AO2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AP2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AQ2" s="7">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:43" ht="16" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:43" ht="15.6">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
@@ -929,7 +995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:43" ht="16" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:43" ht="15.6">
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
@@ -1070,12 +1136,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Hoja2"/>
   <dimension ref="A1:AQ4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="31.6328125" customWidth="1"/>
+    <col min="1" max="1" width="31.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:43" ht="15.6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1206,138 +1272,138 @@
         <v>2060</v>
       </c>
     </row>
-    <row r="2" spans="1:43" ht="16" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:43" ht="15.6">
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="6">
-        <v>0</v>
-      </c>
-      <c r="D2" s="6">
-        <v>0</v>
-      </c>
-      <c r="E2" s="6">
-        <v>0</v>
-      </c>
-      <c r="F2" s="6">
-        <v>0</v>
-      </c>
-      <c r="G2" s="6">
-        <v>0</v>
-      </c>
-      <c r="H2" s="6">
-        <v>0</v>
-      </c>
-      <c r="I2" s="6">
-        <v>0</v>
-      </c>
-      <c r="J2" s="6">
-        <v>0</v>
-      </c>
-      <c r="K2" s="6">
-        <v>0</v>
-      </c>
-      <c r="L2" s="6">
-        <v>0</v>
-      </c>
-      <c r="M2" s="6">
-        <v>0</v>
-      </c>
-      <c r="N2" s="6">
-        <v>0</v>
-      </c>
-      <c r="O2" s="6">
-        <v>0</v>
-      </c>
-      <c r="P2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="6">
-        <v>0</v>
-      </c>
-      <c r="R2" s="6">
-        <v>0</v>
-      </c>
-      <c r="S2" s="6">
-        <v>0</v>
-      </c>
-      <c r="T2" s="6">
-        <v>0</v>
-      </c>
-      <c r="U2" s="6">
-        <v>0</v>
-      </c>
-      <c r="V2" s="6">
-        <v>0</v>
-      </c>
-      <c r="W2" s="6">
-        <v>0</v>
-      </c>
-      <c r="X2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AF2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AG2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AH2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AI2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AJ2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AK2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AL2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AM2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AN2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AO2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AP2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AQ2" s="6">
+      <c r="C2" s="7">
+        <v>0</v>
+      </c>
+      <c r="D2" s="7">
+        <v>0</v>
+      </c>
+      <c r="E2" s="7">
+        <v>0</v>
+      </c>
+      <c r="F2" s="7">
+        <v>0</v>
+      </c>
+      <c r="G2" s="7">
+        <v>0</v>
+      </c>
+      <c r="H2" s="7">
+        <v>0</v>
+      </c>
+      <c r="I2" s="7">
+        <v>0</v>
+      </c>
+      <c r="J2" s="7">
+        <v>0</v>
+      </c>
+      <c r="K2" s="7">
+        <v>0</v>
+      </c>
+      <c r="L2" s="7">
+        <v>0</v>
+      </c>
+      <c r="M2" s="7">
+        <v>0</v>
+      </c>
+      <c r="N2" s="7">
+        <v>0</v>
+      </c>
+      <c r="O2" s="7">
+        <v>0</v>
+      </c>
+      <c r="P2" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="7">
+        <v>0</v>
+      </c>
+      <c r="R2" s="7">
+        <v>0</v>
+      </c>
+      <c r="S2" s="7">
+        <v>0</v>
+      </c>
+      <c r="T2" s="7">
+        <v>0</v>
+      </c>
+      <c r="U2" s="7">
+        <v>0</v>
+      </c>
+      <c r="V2" s="7">
+        <v>0</v>
+      </c>
+      <c r="W2" s="7">
+        <v>0</v>
+      </c>
+      <c r="X2" s="7">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="7">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AD2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AG2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AH2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AI2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AJ2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AK2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AL2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AM2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AN2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AO2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AP2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AQ2" s="7">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:43" ht="16" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:43" ht="15.6">
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
@@ -1468,7 +1534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:43" ht="16" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:43" ht="15.6">
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
@@ -1609,12 +1675,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{916D2B2D-4AA6-4AEC-A74D-5F74F284844E}">
   <sheetPr codeName="Hoja3"/>
   <dimension ref="A1:AQ5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="38.54296875" customWidth="1"/>
+    <col min="1" max="1" width="52.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:43" ht="15.6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1745,400 +1811,400 @@
         <v>2060</v>
       </c>
     </row>
-    <row r="2" spans="1:43" ht="16" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:43" ht="15.6">
       <c r="A2" s="4" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="6">
-        <v>0</v>
-      </c>
-      <c r="D2" s="6">
-        <v>0</v>
-      </c>
-      <c r="E2" s="6">
-        <v>0</v>
-      </c>
-      <c r="F2" s="6">
-        <v>0</v>
-      </c>
-      <c r="G2" s="6">
-        <v>0</v>
-      </c>
-      <c r="H2" s="6">
-        <v>0</v>
-      </c>
-      <c r="I2" s="6">
-        <v>0</v>
-      </c>
-      <c r="J2" s="6">
-        <v>0</v>
-      </c>
-      <c r="K2" s="6">
-        <v>0</v>
-      </c>
-      <c r="L2" s="6">
-        <v>0</v>
-      </c>
-      <c r="M2" s="6">
-        <v>0</v>
-      </c>
-      <c r="N2" s="6">
-        <v>0</v>
-      </c>
-      <c r="O2" s="6">
-        <v>0</v>
-      </c>
-      <c r="P2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="6">
-        <v>0</v>
-      </c>
-      <c r="R2" s="6">
-        <v>0</v>
-      </c>
-      <c r="S2" s="6">
-        <v>0</v>
-      </c>
-      <c r="T2" s="6">
-        <v>0</v>
-      </c>
-      <c r="U2" s="6">
-        <v>0</v>
-      </c>
-      <c r="V2" s="6">
-        <v>0</v>
-      </c>
-      <c r="W2" s="6">
-        <v>0</v>
-      </c>
-      <c r="X2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AB2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AC2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AD2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AF2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AG2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AH2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AI2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AJ2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AK2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AL2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AM2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AN2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AO2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AP2" s="6">
-        <v>0</v>
-      </c>
-      <c r="AQ2" s="6">
+      <c r="C2" s="7">
+        <v>0</v>
+      </c>
+      <c r="D2" s="7">
+        <v>0</v>
+      </c>
+      <c r="E2" s="7">
+        <v>0</v>
+      </c>
+      <c r="F2" s="7">
+        <v>0</v>
+      </c>
+      <c r="G2" s="7">
+        <v>0</v>
+      </c>
+      <c r="H2" s="7">
+        <v>0</v>
+      </c>
+      <c r="I2" s="7">
+        <v>0</v>
+      </c>
+      <c r="J2" s="7">
+        <v>0</v>
+      </c>
+      <c r="K2" s="7">
+        <v>0</v>
+      </c>
+      <c r="L2" s="7">
+        <v>0</v>
+      </c>
+      <c r="M2" s="7">
+        <v>0</v>
+      </c>
+      <c r="N2" s="7">
+        <v>0</v>
+      </c>
+      <c r="O2" s="7">
+        <v>0</v>
+      </c>
+      <c r="P2" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="7">
+        <v>0</v>
+      </c>
+      <c r="R2" s="7">
+        <v>0</v>
+      </c>
+      <c r="S2" s="7">
+        <v>0</v>
+      </c>
+      <c r="T2" s="7">
+        <v>0</v>
+      </c>
+      <c r="U2" s="7">
+        <v>0</v>
+      </c>
+      <c r="V2" s="7">
+        <v>0</v>
+      </c>
+      <c r="W2" s="7">
+        <v>0</v>
+      </c>
+      <c r="X2" s="7">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="7">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AD2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AG2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AH2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AI2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AJ2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AK2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AL2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AM2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AN2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AO2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AP2" s="7">
+        <v>0</v>
+      </c>
+      <c r="AQ2" s="7">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:43" ht="16" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:43" ht="15.6">
       <c r="A3" s="4" t="s">
         <v>8</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="6">
-        <v>0</v>
-      </c>
-      <c r="D3" s="6">
-        <v>0</v>
-      </c>
-      <c r="E3" s="6">
-        <v>0</v>
-      </c>
-      <c r="F3" s="6">
-        <v>0</v>
-      </c>
-      <c r="G3" s="6">
-        <v>0</v>
-      </c>
-      <c r="H3" s="6">
-        <v>0</v>
-      </c>
-      <c r="I3" s="6">
-        <v>0</v>
-      </c>
-      <c r="J3" s="6">
-        <v>0</v>
-      </c>
-      <c r="K3" s="6">
-        <v>0</v>
-      </c>
-      <c r="L3" s="6">
-        <v>0</v>
-      </c>
-      <c r="M3" s="6">
-        <v>0</v>
-      </c>
-      <c r="N3" s="6">
-        <v>0</v>
-      </c>
-      <c r="O3" s="6">
-        <v>0</v>
-      </c>
-      <c r="P3" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="6">
-        <v>0</v>
-      </c>
-      <c r="R3" s="6">
-        <v>0</v>
-      </c>
-      <c r="S3" s="6">
-        <v>0</v>
-      </c>
-      <c r="T3" s="6">
-        <v>0</v>
-      </c>
-      <c r="U3" s="6">
-        <v>0</v>
-      </c>
-      <c r="V3" s="6">
-        <v>0</v>
-      </c>
-      <c r="W3" s="6">
-        <v>0</v>
-      </c>
-      <c r="X3" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y3" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AB3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AC3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AD3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AF3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AG3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AI3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AJ3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AK3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AL3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AM3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AN3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AO3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AP3" s="6">
-        <v>0</v>
-      </c>
-      <c r="AQ3" s="6">
+      <c r="C3" s="7">
+        <v>0</v>
+      </c>
+      <c r="D3" s="7">
+        <v>0</v>
+      </c>
+      <c r="E3" s="7">
+        <v>0</v>
+      </c>
+      <c r="F3" s="7">
+        <v>0</v>
+      </c>
+      <c r="G3" s="7">
+        <v>0</v>
+      </c>
+      <c r="H3" s="7">
+        <v>0</v>
+      </c>
+      <c r="I3" s="7">
+        <v>0</v>
+      </c>
+      <c r="J3" s="7">
+        <v>0</v>
+      </c>
+      <c r="K3" s="7">
+        <v>0</v>
+      </c>
+      <c r="L3" s="7">
+        <v>0</v>
+      </c>
+      <c r="M3" s="7">
+        <v>0</v>
+      </c>
+      <c r="N3" s="7">
+        <v>0</v>
+      </c>
+      <c r="O3" s="7">
+        <v>0</v>
+      </c>
+      <c r="P3" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="7">
+        <v>0</v>
+      </c>
+      <c r="R3" s="7">
+        <v>0</v>
+      </c>
+      <c r="S3" s="7">
+        <v>0</v>
+      </c>
+      <c r="T3" s="7">
+        <v>0</v>
+      </c>
+      <c r="U3" s="7">
+        <v>0</v>
+      </c>
+      <c r="V3" s="7">
+        <v>0</v>
+      </c>
+      <c r="W3" s="7">
+        <v>0</v>
+      </c>
+      <c r="X3" s="7">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="7">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AC3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AD3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AG3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AH3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AI3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AJ3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AK3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AL3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AM3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AN3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AO3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AP3" s="7">
+        <v>0</v>
+      </c>
+      <c r="AQ3" s="7">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:43" ht="16" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:43" ht="15.6">
       <c r="A4" s="4" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="6">
-        <v>0</v>
-      </c>
-      <c r="D4" s="6">
-        <v>0</v>
-      </c>
-      <c r="E4" s="6">
-        <v>0</v>
-      </c>
-      <c r="F4" s="6">
-        <v>0</v>
-      </c>
-      <c r="G4" s="6">
-        <v>0</v>
-      </c>
-      <c r="H4" s="6">
-        <v>0</v>
-      </c>
-      <c r="I4" s="6">
-        <v>0</v>
-      </c>
-      <c r="J4" s="6">
-        <v>0</v>
-      </c>
-      <c r="K4" s="6">
-        <v>0</v>
-      </c>
-      <c r="L4" s="6">
-        <v>0</v>
-      </c>
-      <c r="M4" s="6">
-        <v>0</v>
-      </c>
-      <c r="N4" s="6">
-        <v>0</v>
-      </c>
-      <c r="O4" s="6">
-        <v>0</v>
-      </c>
-      <c r="P4" s="6">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="6">
-        <v>0</v>
-      </c>
-      <c r="R4" s="6">
-        <v>0</v>
-      </c>
-      <c r="S4" s="6">
-        <v>0</v>
-      </c>
-      <c r="T4" s="6">
-        <v>0</v>
-      </c>
-      <c r="U4" s="6">
-        <v>0</v>
-      </c>
-      <c r="V4" s="6">
-        <v>0</v>
-      </c>
-      <c r="W4" s="6">
-        <v>0</v>
-      </c>
-      <c r="X4" s="6">
-        <v>0</v>
-      </c>
-      <c r="Y4" s="6">
-        <v>0</v>
-      </c>
-      <c r="Z4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AA4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AB4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AD4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AE4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AF4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AG4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AH4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AI4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AJ4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AK4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AL4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AM4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AN4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AO4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AP4" s="6">
-        <v>0</v>
-      </c>
-      <c r="AQ4" s="6">
+      <c r="C4" s="7">
+        <v>0</v>
+      </c>
+      <c r="D4" s="7">
+        <v>0</v>
+      </c>
+      <c r="E4" s="7">
+        <v>0</v>
+      </c>
+      <c r="F4" s="7">
+        <v>0</v>
+      </c>
+      <c r="G4" s="7">
+        <v>0</v>
+      </c>
+      <c r="H4" s="7">
+        <v>0</v>
+      </c>
+      <c r="I4" s="7">
+        <v>0</v>
+      </c>
+      <c r="J4" s="7">
+        <v>0</v>
+      </c>
+      <c r="K4" s="7">
+        <v>0</v>
+      </c>
+      <c r="L4" s="7">
+        <v>0</v>
+      </c>
+      <c r="M4" s="7">
+        <v>0</v>
+      </c>
+      <c r="N4" s="7">
+        <v>0</v>
+      </c>
+      <c r="O4" s="7">
+        <v>0</v>
+      </c>
+      <c r="P4" s="7">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="7">
+        <v>0</v>
+      </c>
+      <c r="R4" s="7">
+        <v>0</v>
+      </c>
+      <c r="S4" s="7">
+        <v>0</v>
+      </c>
+      <c r="T4" s="7">
+        <v>0</v>
+      </c>
+      <c r="U4" s="7">
+        <v>0</v>
+      </c>
+      <c r="V4" s="7">
+        <v>0</v>
+      </c>
+      <c r="W4" s="7">
+        <v>0</v>
+      </c>
+      <c r="X4" s="7">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="7">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AF4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AG4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AH4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AI4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AJ4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AK4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AL4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AM4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AN4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AO4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AP4" s="7">
+        <v>0</v>
+      </c>
+      <c r="AQ4" s="7">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="16" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:43" ht="15.6">
       <c r="A5" s="4" t="s">
         <v>11</v>
       </c>
@@ -2148,124 +2214,124 @@
       <c r="C5" s="6">
         <v>0</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="L5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="N5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="O5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="P5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="R5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="S5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="T5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="U5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="V5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="W5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="X5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="Y5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AA5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AB5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AC5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AD5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AE5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AF5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AG5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AH5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AI5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AJ5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AK5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AL5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AM5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AN5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AO5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AP5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="AQ5" s="7" t="s">
+      <c r="D5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="L5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="M5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="N5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="O5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="P5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="R5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="S5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="T5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="U5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="V5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="W5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="X5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AA5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AC5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AD5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AE5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AF5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AG5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AH5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AI5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AJ5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AK5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AL5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AM5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AN5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AO5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AP5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="AQ5" s="10" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>